<commit_message>
Classify 146 exact-name matched education institutions against the 39-school list
</commit_message>
<xml_diff>
--- a/site/exports/bit-physics.xlsx
+++ b/site/exports/bit-physics.xlsx
@@ -742,7 +742,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
@@ -807,7 +807,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr"/>

</xml_diff>